<commit_message>
add noise to data, add accuracy to boruta, compare boruta to xgboost
</commit_message>
<xml_diff>
--- a/podsumowanie_cech_syntetyczne.xlsx
+++ b/podsumowanie_cech_syntetyczne.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kpola\OneDrive\Desktop\Magister\mgst_xgboost\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACE03D2E-294F-4291-9ED0-FC996DBA6192}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB5C2826-3547-4F22-BB4A-113BE84B979B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5535" yWindow="2445" windowWidth="28800" windowHeight="15435" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="17">
   <si>
     <t>XGBOOST</t>
   </si>
@@ -436,16 +436,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="27.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="27.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="23.28515625" bestFit="1" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
@@ -479,58 +471,18 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3">
-        <v>20</v>
-      </c>
-      <c r="C3">
-        <v>18</v>
-      </c>
-      <c r="D3" t="s">
-        <v>5</v>
-      </c>
-      <c r="E3">
-        <v>20</v>
-      </c>
-      <c r="F3">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4">
-        <v>20</v>
-      </c>
-      <c r="C4">
-        <v>15</v>
-      </c>
-      <c r="D4" t="s">
-        <v>6</v>
-      </c>
-      <c r="E4">
-        <v>20</v>
-      </c>
-      <c r="F4">
-        <v>20</v>
-      </c>
-    </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B5">
         <v>20</v>
       </c>
       <c r="C5">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D5" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E5">
         <v>20</v>
@@ -541,188 +493,268 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B6">
         <v>20</v>
       </c>
       <c r="C6">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D6" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E6">
         <v>20</v>
       </c>
       <c r="F6">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B7">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="C7">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="D7" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E7">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="F7">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B8">
+        <v>20</v>
+      </c>
+      <c r="C8">
         <v>13</v>
       </c>
-      <c r="C8">
-        <v>4</v>
-      </c>
       <c r="D8" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E8">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="F8">
-        <v>13</v>
+        <v>19</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B9">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="C9">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D9" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E9">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="F9">
-        <v>0</v>
+        <v>21</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B10">
-        <v>40</v>
+        <v>13</v>
       </c>
       <c r="C10">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D10" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E10">
-        <v>40</v>
+        <v>13</v>
       </c>
       <c r="F10">
-        <v>0</v>
+        <v>13</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B11">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="C11">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D11" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E11">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="F11">
-        <v>16</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B12">
-        <v>7</v>
+        <v>40</v>
       </c>
       <c r="C12">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D12" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E12">
-        <v>7</v>
+        <v>40</v>
       </c>
       <c r="F12">
-        <v>7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B13">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C13">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D13" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E13">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F13">
-        <v>22</v>
+        <v>16</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B14">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="C14">
         <v>2</v>
       </c>
       <c r="D14" t="s">
+        <v>14</v>
+      </c>
+      <c r="E14">
+        <v>7</v>
+      </c>
+      <c r="F14">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>15</v>
+      </c>
+      <c r="B15">
+        <v>22</v>
+      </c>
+      <c r="C15">
+        <v>2</v>
+      </c>
+      <c r="D15" t="s">
+        <v>15</v>
+      </c>
+      <c r="E15">
+        <v>22</v>
+      </c>
+      <c r="F15">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
         <v>16</v>
       </c>
-      <c r="E14">
+      <c r="B16">
         <v>12</v>
       </c>
-      <c r="F14">
+      <c r="C16">
+        <v>2</v>
+      </c>
+      <c r="D16" t="s">
+        <v>16</v>
+      </c>
+      <c r="E16">
         <v>12</v>
+      </c>
+      <c r="F16">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>15</v>
+      </c>
+      <c r="B17">
+        <v>22</v>
+      </c>
+      <c r="C17">
+        <v>2</v>
+      </c>
+      <c r="D17" t="s">
+        <v>15</v>
+      </c>
+      <c r="E17">
+        <v>22</v>
+      </c>
+      <c r="F17">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>15</v>
+      </c>
+      <c r="B18">
+        <v>22</v>
+      </c>
+      <c r="C18">
+        <v>2</v>
+      </c>
+      <c r="D18" t="s">
+        <v>15</v>
+      </c>
+      <c r="E18">
+        <v>22</v>
+      </c>
+      <c r="F18">
+        <v>22</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
     <mergeCell ref="D1:F1"/>
-    <mergeCell ref="A1:C1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>